<commit_message>
All Tests are verified
</commit_message>
<xml_diff>
--- a/Orangehrm.xlsx
+++ b/Orangehrm.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,13 +415,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>' OR '1'='1</v>
+        <v>Admin</v>
       </c>
       <c r="B2" t="str">
         <v>Admin</v>
       </c>
       <c r="C2" t="str">
-        <v>Virat Kohli</v>
+        <v>manda user</v>
       </c>
       <c r="D2" t="str">
         <v>Enabled</v>
@@ -429,13 +429,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ABCCD</v>
+        <v>CKEAi</v>
       </c>
       <c r="B3" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C3" t="str">
-        <v>A8DCo 010Z</v>
+        <v>CKEAi zNnUl</v>
       </c>
       <c r="D3" t="str">
         <v>Enabled</v>
@@ -443,13 +443,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Admin</v>
+        <v>cVZfu</v>
       </c>
       <c r="B4" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C4" t="str">
-        <v>Priyanka Dongare</v>
+        <v>cVZfu EWSzc</v>
       </c>
       <c r="D4" t="str">
         <v>Enabled</v>
@@ -457,13 +457,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Admin1</v>
+        <v>DGwIG</v>
       </c>
       <c r="B5" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C5" t="str">
-        <v>ABC DC</v>
+        <v>DGwIG uCwVE</v>
       </c>
       <c r="D5" t="str">
         <v>Enabled</v>
@@ -471,13 +471,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Afsal123</v>
+        <v>ezuEe</v>
       </c>
       <c r="B6" t="str">
         <v>ESS</v>
       </c>
       <c r="C6" t="str">
-        <v>Afsal f</v>
+        <v>ezuEe kSVud</v>
       </c>
       <c r="D6" t="str">
         <v>Enabled</v>
@@ -485,27 +485,27 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>alex.137391</v>
+        <v>hicksbeverly</v>
       </c>
       <c r="B7" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C7" t="str">
-        <v>Alex137 Hunter391</v>
+        <v>Alexander Baker</v>
       </c>
       <c r="D7" t="str">
-        <v>Enabled</v>
+        <v>Disabled</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>alex.473036</v>
+        <v>jdoe970093</v>
       </c>
       <c r="B8" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C8" t="str">
-        <v>Alex473 Hunter036</v>
+        <v>Jane Doe</v>
       </c>
       <c r="D8" t="str">
         <v>Enabled</v>
@@ -513,13 +513,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Armin</v>
+        <v>Jobinsam@6742</v>
       </c>
       <c r="B9" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C9" t="str">
-        <v>James Butler</v>
+        <v>Jobin Sam</v>
       </c>
       <c r="D9" t="str">
         <v>Enabled</v>
@@ -527,13 +527,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Asmita</v>
+        <v>john321705</v>
       </c>
       <c r="B10" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C10" t="str">
-        <v>Jobin Sam</v>
+        <v>John Doe</v>
       </c>
       <c r="D10" t="str">
         <v>Enabled</v>
@@ -541,13 +541,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Betty19</v>
+        <v>KeARSl</v>
       </c>
       <c r="B11" t="str">
         <v>Admin</v>
       </c>
       <c r="C11" t="str">
-        <v>A8DCo 010Z</v>
+        <v>manda user</v>
       </c>
       <c r="D11" t="str">
         <v>Enabled</v>
@@ -555,13 +555,13 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>chandpatil</v>
+        <v>lIOGZ</v>
       </c>
       <c r="B12" t="str">
         <v>ESS</v>
       </c>
       <c r="C12" t="str">
-        <v>Chandler Patil</v>
+        <v>lIOGZ CqAfp</v>
       </c>
       <c r="D12" t="str">
         <v>Enabled</v>
@@ -569,13 +569,13 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Charles</v>
+        <v>lokesh__11</v>
       </c>
       <c r="B13" t="str">
-        <v>ESS</v>
+        <v>Admin</v>
       </c>
       <c r="C13" t="str">
-        <v>Charles O'Connell</v>
+        <v>yedghjb1 90jsnd</v>
       </c>
       <c r="D13" t="str">
         <v>Enabled</v>
@@ -583,13 +583,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Chetanpawar</v>
+        <v>manju</v>
       </c>
       <c r="B14" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C14" t="str">
-        <v>A8DCo 010Z</v>
+        <v>tabjul manju</v>
       </c>
       <c r="D14" t="str">
         <v>Enabled</v>
@@ -597,13 +597,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>David</v>
+        <v>mohamed.khaled</v>
       </c>
       <c r="B15" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C15" t="str">
-        <v>john Anderson</v>
+        <v>Mohamed Khaled</v>
       </c>
       <c r="D15" t="str">
         <v>Enabled</v>
@@ -611,13 +611,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>deepa</v>
+        <v>NoorRafi0303</v>
       </c>
       <c r="B16" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C16" t="str">
-        <v>Jobin Sam</v>
+        <v>Mohammed Rafi</v>
       </c>
       <c r="D16" t="str">
         <v>Enabled</v>
@@ -625,13 +625,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Edgar66</v>
+        <v>NoorRafi2052</v>
       </c>
       <c r="B17" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C17" t="str">
-        <v>A8DCo 010Z</v>
+        <v>Mohammed Rafi</v>
       </c>
       <c r="D17" t="str">
         <v>Enabled</v>
@@ -639,41 +639,41 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>eKqJR</v>
+        <v>NoorRafi2216</v>
       </c>
       <c r="B18" t="str">
         <v>ESS</v>
       </c>
       <c r="C18" t="str">
-        <v>eKqJR BBOnw</v>
+        <v>Mohammed Rafi</v>
       </c>
       <c r="D18" t="str">
-        <v>Enabled</v>
+        <v>Disabled</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ElianaBabirye2</v>
+        <v>NoorRafi3339</v>
       </c>
       <c r="B19" t="str">
         <v>ESS</v>
       </c>
       <c r="C19" t="str">
-        <v>Eliana Nakyeyune</v>
+        <v>Mohammed Rafi</v>
       </c>
       <c r="D19" t="str">
-        <v>Enabled</v>
+        <v>Disabled</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Evan16</v>
+        <v>NoorRafi4063</v>
       </c>
       <c r="B20" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C20" t="str">
-        <v>A8DCo 010Z</v>
+        <v>Mohammed Rafi</v>
       </c>
       <c r="D20" t="str">
         <v>Enabled</v>
@@ -681,13 +681,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>FMLName</v>
+        <v>NoorRafi6619</v>
       </c>
       <c r="B21" t="str">
         <v>ESS</v>
       </c>
       <c r="C21" t="str">
-        <v>Qwerty LName</v>
+        <v>Mohammed Rafi</v>
       </c>
       <c r="D21" t="str">
         <v>Enabled</v>
@@ -695,13 +695,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>FMLName1</v>
+        <v>NoorRafi9607</v>
       </c>
       <c r="B22" t="str">
         <v>ESS</v>
       </c>
       <c r="C22" t="str">
-        <v>FName LName</v>
+        <v>Mohammed Rafi</v>
       </c>
       <c r="D22" t="str">
         <v>Enabled</v>
@@ -709,13 +709,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>FxPMf</v>
+        <v>RJspi</v>
       </c>
       <c r="B23" t="str">
         <v>ESS</v>
       </c>
       <c r="C23" t="str">
-        <v>FxPMf cGfgQ</v>
+        <v>RJspi FKRSv</v>
       </c>
       <c r="D23" t="str">
         <v>Enabled</v>
@@ -723,13 +723,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Gauriii</v>
+        <v>Rosanna</v>
       </c>
       <c r="B24" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C24" t="str">
-        <v>Priyanka Dongare</v>
+        <v>Rosanna Pagac</v>
       </c>
       <c r="D24" t="str">
         <v>Enabled</v>
@@ -737,13 +737,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>gokua2f0ba1f-f005-4eee-9aac-8552216e486d</v>
+        <v>Rudzani@123</v>
       </c>
       <c r="B25" t="str">
         <v>ESS</v>
       </c>
       <c r="C25" t="str">
-        <v>Qwerty LName</v>
+        <v>Peter Anderson</v>
       </c>
       <c r="D25" t="str">
         <v>Enabled</v>
@@ -751,13 +751,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Harshali</v>
+        <v>Savina1234</v>
       </c>
       <c r="B26" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C26" t="str">
-        <v>A8DCo 010Z</v>
+        <v>savina dulvin</v>
       </c>
       <c r="D26" t="str">
         <v>Enabled</v>
@@ -765,13 +765,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>HhSSV</v>
+        <v>shortstephanie</v>
       </c>
       <c r="B27" t="str">
         <v>ESS</v>
       </c>
       <c r="C27" t="str">
-        <v>HhSSV xGxpO</v>
+        <v>Joseph Thomas</v>
       </c>
       <c r="D27" t="str">
         <v>Enabled</v>
@@ -779,13 +779,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Janhavi</v>
+        <v>Tabjul</v>
       </c>
       <c r="B28" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C28" t="str">
-        <v>James Butler</v>
+        <v>Manju Tabjul</v>
       </c>
       <c r="D28" t="str">
         <v>Enabled</v>
@@ -793,27 +793,27 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>JeDFX</v>
+        <v>test0714</v>
       </c>
       <c r="B29" t="str">
         <v>ESS</v>
       </c>
       <c r="C29" t="str">
-        <v>JeDFX yGxJt</v>
+        <v>Test Employee1784109636</v>
       </c>
       <c r="D29" t="str">
-        <v>Enabled</v>
+        <v>Disabled</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Jobinsam@6742</v>
+        <v>VQdEmc</v>
       </c>
       <c r="B30" t="str">
-        <v>ESS</v>
+        <v>Admin</v>
       </c>
       <c r="C30" t="str">
-        <v>Jobin Sam</v>
+        <v>manda user</v>
       </c>
       <c r="D30" t="str">
         <v>Enabled</v>
@@ -821,301 +821,21 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>joeyshah</v>
+        <v>xyz.abc</v>
       </c>
       <c r="B31" t="str">
         <v>Admin</v>
       </c>
       <c r="C31" t="str">
-        <v>Joey Shah</v>
+        <v>xyz abc</v>
       </c>
       <c r="D31" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>john123456</v>
-      </c>
-      <c r="B32" t="str">
-        <v>Admin</v>
-      </c>
-      <c r="C32" t="str">
-        <v>john Anderson</v>
-      </c>
-      <c r="D32" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>john1234565</v>
-      </c>
-      <c r="B33" t="str">
-        <v>Admin</v>
-      </c>
-      <c r="C33" t="str">
-        <v>john Anderson</v>
-      </c>
-      <c r="D33" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>john402732</v>
-      </c>
-      <c r="B34" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C34" t="str">
-        <v>John Doe</v>
-      </c>
-      <c r="D34" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>johndoe_test01</v>
-      </c>
-      <c r="B35" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C35" t="str">
-        <v>John Doe</v>
-      </c>
-      <c r="D35" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>Julio95</v>
-      </c>
-      <c r="B36" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C36" t="str">
-        <v>A8DCo 010Z</v>
-      </c>
-      <c r="D36" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>L1_test044022</v>
-      </c>
-      <c r="B37" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C37" t="str">
-        <v>L1 Track</v>
-      </c>
-      <c r="D37" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>Manasvi</v>
-      </c>
-      <c r="B38" t="str">
-        <v>Admin</v>
-      </c>
-      <c r="C38" t="str">
-        <v>Ravi B</v>
-      </c>
-      <c r="D38" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>mismatchUser_248392</v>
-      </c>
-      <c r="B39" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C39" t="str">
-        <v>Reza Kareem</v>
-      </c>
-      <c r="D39" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>mismatchUser_563546</v>
-      </c>
-      <c r="B40" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C40" t="str">
-        <v>Reza Kareem</v>
-      </c>
-      <c r="D40" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>mismatchUser_566725</v>
-      </c>
-      <c r="B41" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C41" t="str">
-        <v>Reza Kareem</v>
-      </c>
-      <c r="D41" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>MMzYP</v>
-      </c>
-      <c r="B42" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C42" t="str">
-        <v>MMzYP LnVRL</v>
-      </c>
-      <c r="D42" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>newemployee</v>
-      </c>
-      <c r="B43" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C43" t="str">
-        <v>CalibreQA 1784090449548</v>
-      </c>
-      <c r="D43" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v>nilam swapnil</v>
-      </c>
-      <c r="B44" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C44" t="str">
-        <v>john Anderson</v>
-      </c>
-      <c r="D44" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="str">
-        <v>NoorRafi2650</v>
-      </c>
-      <c r="B45" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C45" t="str">
-        <v>Mohammed Rafi</v>
-      </c>
-      <c r="D45" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>NoorRafi3215</v>
-      </c>
-      <c r="B46" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C46" t="str">
-        <v>Mohammed Rafi</v>
-      </c>
-      <c r="D46" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>NoorRafi4107</v>
-      </c>
-      <c r="B47" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C47" t="str">
-        <v>Mohammed Rafi</v>
-      </c>
-      <c r="D47" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>NoorRafi7265</v>
-      </c>
-      <c r="B48" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C48" t="str">
-        <v>Mohammed Rafi</v>
-      </c>
-      <c r="D48" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>NoorRafi7607</v>
-      </c>
-      <c r="B49" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C49" t="str">
-        <v>Mohammed Rafi</v>
-      </c>
-      <c r="D49" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
-        <v>NoorRafi7707</v>
-      </c>
-      <c r="B50" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C50" t="str">
-        <v>Mohammed Rafi</v>
-      </c>
-      <c r="D50" t="str">
-        <v>Enabled</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>NoorRafi8941</v>
-      </c>
-      <c r="B51" t="str">
-        <v>ESS</v>
-      </c>
-      <c r="C51" t="str">
-        <v>Mohammed Rafi</v>
-      </c>
-      <c r="D51" t="str">
         <v>Enabled</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Test are reflected to be slow
</commit_message>
<xml_diff>
--- a/Orangehrm.xlsx
+++ b/Orangehrm.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D50"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,13 +429,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>CKEAi</v>
+        <v>Admin1234567</v>
       </c>
       <c r="B3" t="str">
-        <v>ESS</v>
+        <v>Admin</v>
       </c>
       <c r="C3" t="str">
-        <v>CKEAi zNnUl</v>
+        <v>new test employee</v>
       </c>
       <c r="D3" t="str">
         <v>Enabled</v>
@@ -443,13 +443,13 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>cVZfu</v>
+        <v>anu02</v>
       </c>
       <c r="B4" t="str">
         <v>ESS</v>
       </c>
       <c r="C4" t="str">
-        <v>cVZfu EWSzc</v>
+        <v>Anu George</v>
       </c>
       <c r="D4" t="str">
         <v>Enabled</v>
@@ -457,13 +457,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>DGwIG</v>
+        <v>arun05</v>
       </c>
       <c r="B5" t="str">
         <v>ESS</v>
       </c>
       <c r="C5" t="str">
-        <v>DGwIG uCwVE</v>
+        <v>Arun Kumar</v>
       </c>
       <c r="D5" t="str">
         <v>Enabled</v>
@@ -471,13 +471,13 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ezuEe</v>
+        <v>CKEAi</v>
       </c>
       <c r="B6" t="str">
         <v>ESS</v>
       </c>
       <c r="C6" t="str">
-        <v>ezuEe kSVud</v>
+        <v>CKEAi zNnUl</v>
       </c>
       <c r="D6" t="str">
         <v>Enabled</v>
@@ -485,27 +485,27 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>hicksbeverly</v>
+        <v>cVZfu</v>
       </c>
       <c r="B7" t="str">
         <v>ESS</v>
       </c>
       <c r="C7" t="str">
-        <v>Alexander Baker</v>
+        <v>cVZfu EWSzc</v>
       </c>
       <c r="D7" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>jdoe970093</v>
+        <v>DGwIG</v>
       </c>
       <c r="B8" t="str">
         <v>ESS</v>
       </c>
       <c r="C8" t="str">
-        <v>Jane Doe</v>
+        <v>DGwIG uCwVE</v>
       </c>
       <c r="D8" t="str">
         <v>Enabled</v>
@@ -513,13 +513,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Jobinsam@6742</v>
+        <v>EfqqJX</v>
       </c>
       <c r="B9" t="str">
-        <v>ESS</v>
+        <v>Admin</v>
       </c>
       <c r="C9" t="str">
-        <v>Jobin Sam</v>
+        <v>manda user</v>
       </c>
       <c r="D9" t="str">
         <v>Enabled</v>
@@ -527,13 +527,13 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>john321705</v>
+        <v>eVBqg</v>
       </c>
       <c r="B10" t="str">
         <v>ESS</v>
       </c>
       <c r="C10" t="str">
-        <v>John Doe</v>
+        <v>eVBqg EBTon</v>
       </c>
       <c r="D10" t="str">
         <v>Enabled</v>
@@ -541,13 +541,13 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>KeARSl</v>
+        <v>ezuEe</v>
       </c>
       <c r="B11" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C11" t="str">
-        <v>manda user</v>
+        <v>ezuEe kSVud</v>
       </c>
       <c r="D11" t="str">
         <v>Enabled</v>
@@ -555,13 +555,13 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>lIOGZ</v>
+        <v>gyEViJ</v>
       </c>
       <c r="B12" t="str">
-        <v>ESS</v>
+        <v>Admin</v>
       </c>
       <c r="C12" t="str">
-        <v>lIOGZ CqAfp</v>
+        <v>manda user</v>
       </c>
       <c r="D12" t="str">
         <v>Enabled</v>
@@ -569,27 +569,27 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>lokesh__11</v>
+        <v>hicksbeverly</v>
       </c>
       <c r="B13" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C13" t="str">
-        <v>yedghjb1 90jsnd</v>
+        <v>Alexander Baker</v>
       </c>
       <c r="D13" t="str">
-        <v>Enabled</v>
+        <v>Disabled</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>manju</v>
+        <v>HsOcE</v>
       </c>
       <c r="B14" t="str">
         <v>ESS</v>
       </c>
       <c r="C14" t="str">
-        <v>tabjul manju</v>
+        <v>HsOcE WkjGO</v>
       </c>
       <c r="D14" t="str">
         <v>Enabled</v>
@@ -597,13 +597,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>mohamed.khaled</v>
+        <v>jdoe970093</v>
       </c>
       <c r="B15" t="str">
         <v>ESS</v>
       </c>
       <c r="C15" t="str">
-        <v>Mohamed Khaled</v>
+        <v>Jane Doe</v>
       </c>
       <c r="D15" t="str">
         <v>Enabled</v>
@@ -611,13 +611,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>NoorRafi0303</v>
+        <v>Jobinsam@6742</v>
       </c>
       <c r="B16" t="str">
         <v>ESS</v>
       </c>
       <c r="C16" t="str">
-        <v>Mohammed Rafi</v>
+        <v>Jobin Sam</v>
       </c>
       <c r="D16" t="str">
         <v>Enabled</v>
@@ -625,13 +625,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>NoorRafi2052</v>
+        <v>john01</v>
       </c>
       <c r="B17" t="str">
         <v>ESS</v>
       </c>
       <c r="C17" t="str">
-        <v>Mohammed Rafi</v>
+        <v>John Thomas</v>
       </c>
       <c r="D17" t="str">
         <v>Enabled</v>
@@ -639,41 +639,41 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>NoorRafi2216</v>
+        <v>john321705</v>
       </c>
       <c r="B18" t="str">
         <v>ESS</v>
       </c>
       <c r="C18" t="str">
-        <v>Mohammed Rafi</v>
+        <v>John Doe</v>
       </c>
       <c r="D18" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>NoorRafi3339</v>
+        <v>John_1234</v>
       </c>
       <c r="B19" t="str">
-        <v>ESS</v>
+        <v>Admin</v>
       </c>
       <c r="C19" t="str">
-        <v>Mohammed Rafi</v>
+        <v>John Automation</v>
       </c>
       <c r="D19" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>NoorRafi4063</v>
+        <v>KeARSl</v>
       </c>
       <c r="B20" t="str">
-        <v>ESS</v>
+        <v>Admin</v>
       </c>
       <c r="C20" t="str">
-        <v>Mohammed Rafi</v>
+        <v>manda user</v>
       </c>
       <c r="D20" t="str">
         <v>Enabled</v>
@@ -681,13 +681,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>NoorRafi6619</v>
+        <v>kGMCT</v>
       </c>
       <c r="B21" t="str">
         <v>ESS</v>
       </c>
       <c r="C21" t="str">
-        <v>Mohammed Rafi</v>
+        <v>kGMCT IzDjI</v>
       </c>
       <c r="D21" t="str">
         <v>Enabled</v>
@@ -695,13 +695,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>NoorRafi9607</v>
+        <v>kumarxyz</v>
       </c>
       <c r="B22" t="str">
         <v>ESS</v>
       </c>
       <c r="C22" t="str">
-        <v>Mohammed Rafi</v>
+        <v>KASARAMONI KUMAR</v>
       </c>
       <c r="D22" t="str">
         <v>Enabled</v>
@@ -709,13 +709,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>RJspi</v>
+        <v>lIOGZ</v>
       </c>
       <c r="B23" t="str">
         <v>ESS</v>
       </c>
       <c r="C23" t="str">
-        <v>RJspi FKRSv</v>
+        <v>lIOGZ CqAfp</v>
       </c>
       <c r="D23" t="str">
         <v>Enabled</v>
@@ -723,13 +723,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Rosanna</v>
+        <v>lokesh__11</v>
       </c>
       <c r="B24" t="str">
-        <v>ESS</v>
+        <v>Admin</v>
       </c>
       <c r="C24" t="str">
-        <v>Rosanna Pagac</v>
+        <v>yedghjb1 90jsnd</v>
       </c>
       <c r="D24" t="str">
         <v>Enabled</v>
@@ -737,13 +737,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Rudzani@123</v>
+        <v>manju</v>
       </c>
       <c r="B25" t="str">
         <v>ESS</v>
       </c>
       <c r="C25" t="str">
-        <v>Peter Anderson</v>
+        <v>tabjul manju</v>
       </c>
       <c r="D25" t="str">
         <v>Enabled</v>
@@ -751,13 +751,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Savina1234</v>
+        <v>mohamed.khaled</v>
       </c>
       <c r="B26" t="str">
         <v>ESS</v>
       </c>
       <c r="C26" t="str">
-        <v>savina dulvin</v>
+        <v>Mohamed Khaled</v>
       </c>
       <c r="D26" t="str">
         <v>Enabled</v>
@@ -765,13 +765,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>shortstephanie</v>
+        <v>nisss</v>
       </c>
       <c r="B27" t="str">
-        <v>ESS</v>
+        <v>Admin</v>
       </c>
       <c r="C27" t="str">
-        <v>Joseph Thomas</v>
+        <v>yedghjb1 90jsnd</v>
       </c>
       <c r="D27" t="str">
         <v>Enabled</v>
@@ -779,13 +779,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Tabjul</v>
+        <v>NoorRafi0303</v>
       </c>
       <c r="B28" t="str">
         <v>ESS</v>
       </c>
       <c r="C28" t="str">
-        <v>Manju Tabjul</v>
+        <v>Mohammed Rafi</v>
       </c>
       <c r="D28" t="str">
         <v>Enabled</v>
@@ -793,27 +793,27 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>test0714</v>
+        <v>NoorRafi1868</v>
       </c>
       <c r="B29" t="str">
         <v>ESS</v>
       </c>
       <c r="C29" t="str">
-        <v>Test Employee1784109636</v>
+        <v>Mohammed Rafi</v>
       </c>
       <c r="D29" t="str">
-        <v>Disabled</v>
+        <v>Enabled</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>VQdEmc</v>
+        <v>NoorRafi2052</v>
       </c>
       <c r="B30" t="str">
-        <v>Admin</v>
+        <v>ESS</v>
       </c>
       <c r="C30" t="str">
-        <v>manda user</v>
+        <v>Mohammed Rafi</v>
       </c>
       <c r="D30" t="str">
         <v>Enabled</v>
@@ -821,21 +821,287 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
+        <v>NoorRafi2216</v>
+      </c>
+      <c r="B31" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Mohammed Rafi</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Disabled</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>NoorRafi3339</v>
+      </c>
+      <c r="B32" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Mohammed Rafi</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Disabled</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>NoorRafi4063</v>
+      </c>
+      <c r="B33" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Mohammed Rafi</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>NoorRafi6619</v>
+      </c>
+      <c r="B34" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Mohammed Rafi</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>NoorRafi8372</v>
+      </c>
+      <c r="B35" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Mohammed Rafi</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>NoorRafi8379</v>
+      </c>
+      <c r="B36" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Mohammed Rafi</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>NoorRafi9607</v>
+      </c>
+      <c r="B37" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Mohammed Rafi</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>priya04</v>
+      </c>
+      <c r="B38" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Priya Menon</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Disabled</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>rahul03</v>
+      </c>
+      <c r="B39" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Rahul Nair</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>RJspi</v>
+      </c>
+      <c r="B40" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C40" t="str">
+        <v>RJspi FKRSv</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Rocky007</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Lila Abernathy</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Rosanna</v>
+      </c>
+      <c r="B42" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Rosanna Pagac</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Rudzani@123</v>
+      </c>
+      <c r="B43" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Peter Anderson</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Savina1234</v>
+      </c>
+      <c r="B44" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C44" t="str">
+        <v>savina dulvin</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>shortstephanie</v>
+      </c>
+      <c r="B45" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Joseph Thomas</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Tabjul</v>
+      </c>
+      <c r="B46" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Manju Tabjul</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>test0714</v>
+      </c>
+      <c r="B47" t="str">
+        <v>ESS</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Test Employee1784109636</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>vheodB</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="C48" t="str">
+        <v>manda user</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>VQdEmc</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="C49" t="str">
+        <v>manda user</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Enabled</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
         <v>xyz.abc</v>
       </c>
-      <c r="B31" t="str">
-        <v>Admin</v>
-      </c>
-      <c r="C31" t="str">
+      <c r="B50" t="str">
+        <v>Admin</v>
+      </c>
+      <c r="C50" t="str">
         <v>xyz abc</v>
       </c>
-      <c r="D31" t="str">
+      <c r="D50" t="str">
         <v>Enabled</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D50"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>